<commit_message>
Store calibration history in JSON and preserve run-outs outside fitting
Recovered local commit 3f9fb648aeb444cfd3ec6a06bd4fc308559390f8.
</commit_message>
<xml_diff>
--- a/Experimental_Data/42CrMo4_QT.xlsx
+++ b/Experimental_Data/42CrMo4_QT.xlsx
@@ -3075,9 +3075,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EB9CA7B-F9F7-4B65-BAF9-0554C4DD3A3C}" name="Tabella1" displayName="Tabella1" ref="A1:R5" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
-  <autoFilter ref="A1:R5" xr:uid="{7EB9CA7B-F9F7-4B65-BAF9-0554C4DD3A3C}"/>
-  <tableColumns count="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EB9CA7B-F9F7-4B65-BAF9-0554C4DD3A3C}" name="Tabella1" displayName="Tabella1" ref="A1:K5" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+  <autoFilter ref="A1:K5" xr:uid="{7EB9CA7B-F9F7-4B65-BAF9-0554C4DD3A3C}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{8E3D1E9D-FBEE-441F-8710-5037CD4F23F4}" name="Article DOI" dataDxfId="54"/>
     <tableColumn id="11" xr3:uid="{DB748F3A-E0FD-40A7-AD76-C03A14000D6D}" name="Authors" dataDxfId="53"/>
     <tableColumn id="8" xr3:uid="{5AA73CAD-51B7-41DD-94EB-F60F774B9687}" name="Article year" dataDxfId="52"/>
@@ -3091,13 +3091,6 @@
     <tableColumn id="10" xr3:uid="{EC242BA9-DE01-42A2-8C6C-75459CDE529E}" name="K" dataDxfId="44">
       <calculatedColumnFormula>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit* (MPa)]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{2706D70E-07F0-46AE-B060-716EFEF46FE9}" name="k FS (-)" dataDxfId="43"/>
-    <tableColumn id="13" xr3:uid="{AC0C9453-4F1D-428E-8B4A-FFA7F59C8629}" name="k FI (-)" dataDxfId="42"/>
-    <tableColumn id="14" xr3:uid="{EA69BACE-38CD-4848-A951-727183E325BD}" name="L_LI" dataDxfId="41"/>
-    <tableColumn id="15" xr3:uid="{AD38DCC0-5477-4850-A1CD-A527B66FD54B}" name="k_MGSE" dataDxfId="40"/>
-    <tableColumn id="16" xr3:uid="{93701C45-3072-4892-A612-86238225891A}" name="a_MSWT" dataDxfId="39"/>
-    <tableColumn id="17" xr3:uid="{AE589AEA-A7D1-4655-B471-D0348982CA47}" name="alpha_w" dataDxfId="38"/>
-    <tableColumn id="18" xr3:uid="{AE7D108F-3C88-417B-A3AE-99FBE587FFDD}" name="xi_ZHU" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3513,27 +3506,6 @@
       <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>192</v>
-      </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3570,27 +3542,6 @@
         <f>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit* (MPa)]]))</f>
         <v>Null</v>
       </c>
-      <c r="L2" s="1">
-        <v>2.0699999999999998</v>
-      </c>
-      <c r="M2" s="1">
-        <v>0.83</v>
-      </c>
-      <c r="N2" s="1">
-        <v>5</v>
-      </c>
-      <c r="O2" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="P2" s="1">
-        <v>0.53</v>
-      </c>
-      <c r="Q2" s="1">
-        <v>0</v>
-      </c>
-      <c r="R2" s="1">
-        <v>1</v>
-      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -3627,27 +3578,6 @@
         <f>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit* (MPa)]]))</f>
         <v>1.2587209302325582</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -3684,27 +3614,6 @@
         <f>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit* (MPa)]]))</f>
         <v>Null</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="5" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -3740,27 +3649,6 @@
       <c r="K5" s="1" t="str">
         <f>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]:[Torsional fatigue limit* (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit* (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit* (MPa)]]))</f>
         <v>Null</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -3798,34 +3686,6 @@
         <f>IF(COUNT(Tabella1[K])=0, "Null", AVERAGE(Tabella1[K]))</f>
         <v>1.2587209302325582</v>
       </c>
-      <c r="L6" s="4">
-        <f>IF(COUNT(Tabella1[k FS (-)])=0, "Null", AVERAGE(Tabella1[k FS (-)]))</f>
-        <v>2.0699999999999998</v>
-      </c>
-      <c r="M6" s="4">
-        <f>IF(COUNT(Tabella1[k FI (-)])=0, "Null", AVERAGE(Tabella1[k FI (-)]))</f>
-        <v>0.83</v>
-      </c>
-      <c r="N6" s="4">
-        <f>IF(COUNT(Tabella1[L_LI])=0, "Null", AVERAGE(Tabella1[L_LI]))</f>
-        <v>5</v>
-      </c>
-      <c r="O6" s="4">
-        <f>IF(COUNT(Tabella1[k_MGSE])=0, "Null", AVERAGE(Tabella1[k_MGSE]))</f>
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="P6" s="4">
-        <f>IF(COUNT(Tabella1[a_MSWT])=0, "Null", AVERAGE(Tabella1[a_MSWT]))</f>
-        <v>0.53</v>
-      </c>
-      <c r="Q6" s="4">
-        <f>IF(COUNT(Tabella1[alpha_w])=0, "Null", AVERAGE(Tabella1[alpha_w]))</f>
-        <v>0</v>
-      </c>
-      <c r="R6" s="4">
-        <f>IF(COUNT(Tabella1[xi_ZHU])=0, "Null", AVERAGE(Tabella1[xi_ZHU]))</f>
-        <v>1</v>
-      </c>
     </row>
     <row r="7" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
@@ -3859,34 +3719,6 @@
       </c>
       <c r="K7" s="6">
         <f>IF(COUNT(Tabella1[K])=0, "Null", _xlfn.STDEV.P(Tabella1[K]))</f>
-        <v>0</v>
-      </c>
-      <c r="L7" s="6">
-        <f>IF(COUNT(Tabella1[k FS (-)])=0, "Null", _xlfn.STDEV.P(Tabella1[k FS (-)]))</f>
-        <v>0</v>
-      </c>
-      <c r="M7" s="6">
-        <f>IF(COUNT(Tabella1[k FI (-)])=0, "Null", _xlfn.STDEV.P(Tabella1[k FI (-)]))</f>
-        <v>0</v>
-      </c>
-      <c r="N7" s="6">
-        <f>IF(COUNT(Tabella1[L_LI])=0, "Null", _xlfn.STDEV.P(Tabella1[L_LI]))</f>
-        <v>0</v>
-      </c>
-      <c r="O7" s="6">
-        <f>IF(COUNT(Tabella1[k_MGSE])=0, "Null", _xlfn.STDEV.P(Tabella1[k_MGSE]))</f>
-        <v>0</v>
-      </c>
-      <c r="P7" s="6">
-        <f>IF(COUNT(Tabella1[a_MSWT])=0, "Null", _xlfn.STDEV.P(Tabella1[a_MSWT]))</f>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="6">
-        <f>IF(COUNT(Tabella1[alpha_w])=0, "Null", _xlfn.STDEV.P(Tabella1[alpha_w]))</f>
-        <v>0</v>
-      </c>
-      <c r="R7" s="6">
-        <f>IF(COUNT(Tabella1[xi_ZHU])=0, "Null", _xlfn.STDEV.P(Tabella1[xi_ZHU]))</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>